<commit_message>
Add 12 source-reviewed Tianjin University profiles with conservative evidence and append conservation
</commit_message>
<xml_diff>
--- a/site/exports/tju-math.xlsx
+++ b/site/exports/tju-math.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>数学学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Independent directory and current employment unverified; official university biography supports partial facts only.；Degree labels and study endpoints do not independently establish awards or award dates.；Own mentor names not retained; own supervisor title does not establish who supervised this person.；Bibliographic details are source-reported only; full texts, publisher records and DOI registry not authenticated.；Displayed page date is not a verified update time; source present-tense appointments are not realtime personnel certification.；Displayed 2019 date coexists with source-reported 2024 work; neither authenticates last update.；当前人事状态未知、现职导航关闭；保留来源历史职称与任期，不把导师资格当本人师承。；只采纳必要职业摘录，未核原始学位证、论文、出版者元数据或全文。；院系法定行政父级、校区及院校985地域分类未另核；不补层级。；独立教师目录与当前人事未核，仅官网人物资料支持partial；学历标签和学习终点不证明明确授位。；整理保留原摘录空白规范化与身份字段分隔符添加，不声称原HTTP字节准确复制。；页面显示日期不代表最后更新；原至今职业任期不独立证明现职。；页面显示2019-06-03 00:23与正文2024作品并存，不据此认证更新时间。两篇with合作者不是完整作者顺序；2023 online first与DOI仅原书目。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2164,8 +2218,394 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>degree_study</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>河北工业大学</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2000-09</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2004-06</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>学习标签与起止不证明授位；非学位经历false是事件分类，不否认本人资格。</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>degree_study</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2004-09</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2007-03</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>学习标签与起止不证明授位；非学位经历false是事件分类，不否认本人资格。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>degree_study</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2007-03</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2010-03</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>学习标签与起止不证明授位；非学位经历false是事件分类，不否认本人资格。</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>visiting_scholar</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>访问学者</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>巴斯克应用数学中心(西班牙)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2015-03</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2016-03</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>学习标签与起止不证明授位；非学位经历false是事件分类，不否认本人资格。</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>visiting_scholar</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>访问学者</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>明尼苏达大学德卢斯分校(美国)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2017-08</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2017-10</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>学习标签与起止不证明授位；非学位经历false是事件分类，不否认本人资格。</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>教授、博导</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>天津大学数学学院</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2020-06</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>来源职业角色与原任期保留；至今或未列日期不证明观察日仍任职。</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S20"/>
+  <autoFilter ref="A1:S26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -2186,6 +2626,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2288,7 +2734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2296,11 +2742,11 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="60.2" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="39.2" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -2535,8 +2981,120 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Stabilization for wave equation with localized Kelvin-Voigt damping on cuboidal domain: A degenerate case</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（官网书目）；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目；未核出版元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>原作者/合作者与书目元数据按来源保留，未独立核出版记录。</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>韩忠杰</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Saturated boundary feedback stabilization for a non-uniform Timoshenko beam with disturbances and uncertainties</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文（官网书目）；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目；未核出版元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>原作者/合作者与书目元数据按来源保留，未独立核出版记录。来源年份2023、online first及DOI未作外部认证；with合作者不作完整作者列表。</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L4"/>
+  <autoFilter ref="A1:L6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2547,6 +3105,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2558,7 +3122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2943,27 +3507,23 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>鲍建海</t>
+          <t>韩忠杰</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-3</t>
+          <t>tju-hanzhongjie-profile</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>https://www.csu.edu.cn/zjzn/xxgk.htm</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
-        </is>
-      </c>
+          <t>https://math.tju.edu.cn/info/1715/5554.htm</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2980,7 +3540,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>曹杰</t>
+          <t>鲍建海</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2990,7 +3550,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>https://www.jlu.edu.cn/xxgk.htm</t>
+          <t>https://www.csu.edu.cn/zjzn/xxgk.htm</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3022,37 +3582,74 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>institution-classification-3</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jlu.edu.cn/xxgk.htm</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>天津大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>曹杰</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
           <t>institution-classification-4</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>https://www.csust.edu.cn/fzgh/info/1016/1662.htm</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>tju</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>tju</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>天津大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -3066,6 +3663,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>